<commit_message>
Simplify assessment narrative and add review visuals
</commit_message>
<xml_diff>
--- a/deliverables/Amazon_Q2_2026_Profitability_Analysis.xlsx
+++ b/deliverables/Amazon_Q2_2026_Profitability_Analysis.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rbbfca47753f94184"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Profitability" sheetId="2" r:id="Racc5228479af42b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKU Profitability" sheetId="3" r:id="R7270b48d13094794"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory Health" sheetId="4" r:id="R388ae878c70840ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQ &amp; Assumptions" sheetId="5" r:id="Rdc2184c8c7bb4825"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PO Unit Costs" sheetId="6" r:id="Rfcfd3e285ada42b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="7" r:id="Rd8be4902e3484600"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R43576ba2c2d2418e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Profitability" sheetId="2" r:id="R2079f288094f490b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKU Profitability" sheetId="3" r:id="R82114d1812d5459a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory Health" sheetId="4" r:id="Rccedbad2bf044ab2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQ &amp; Assumptions" sheetId="5" r:id="R296876f5914a4c97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PO Unit Costs" sheetId="6" r:id="R4a422f2adc6f4bea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="7" r:id="Rb9cdfe3e79be41ed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -618,7 +618,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcaf1380107a24e09"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0798236d84c44e60"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -639,7 +639,7 @@
     <x:tableColumn id="7" name="Net Units"/>
     <x:tableColumn id="8" name="Landed COGS"/>
     <x:tableColumn id="9" name="Contribution Margin"/>
-    <x:tableColumn id="10" name="CM %"/>
+    <x:tableColumn id="10" name="Margin %"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -661,7 +661,7 @@
     <x:tableColumn id="11" name="Cost Status"/>
     <x:tableColumn id="12" name="Landed COGS"/>
     <x:tableColumn id="13" name="Contribution Margin"/>
-    <x:tableColumn id="14" name="CM %"/>
+    <x:tableColumn id="14" name="Margin %"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -977,12 +977,12 @@
       <x:c r="E5" s="48"/>
       <x:c r="F5" s="49"/>
       <x:c r="G5" s="47" t="str">
-        <x:v>CM %</x:v>
+        <x:v>MARGIN %</x:v>
       </x:c>
       <x:c r="H5" s="48"/>
       <x:c r="I5" s="49"/>
       <x:c r="J5" s="47" t="str">
-        <x:v>AFTER PLATFORM OVERHEAD</x:v>
+        <x:v>AFTER PLATFORM COSTS</x:v>
       </x:c>
       <x:c r="K5" s="48"/>
     </x:row>
@@ -1049,10 +1049,10 @@
         <x:v>COGS</x:v>
       </x:c>
       <x:c r="I10" s="13" t="str">
-        <x:v>CM</x:v>
+        <x:v>Contribution</x:v>
       </x:c>
       <x:c r="J10" s="14" t="str">
-        <x:v>CM %</x:v>
+        <x:v>Margin %</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1190,7 +1190,7 @@
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="37" t="str">
-        <x:v>1. Protect profitable demand: Peak Fuel and GlowTheory generate 83% of CM1; GT-SERUM-VITC and PF-WHEY-CHOC are the largest SKU contributors.</x:v>
+        <x:v>1. Protect profitable demand: Peak Fuel and GlowTheory generate 83% of contribution margin; GT-SERUM-VITC and PF-WHEY-CHOC are the largest SKU contributors.</x:v>
       </x:c>
       <x:c r="B17" s="37"/>
       <x:c r="C17" s="37"/>
@@ -1200,7 +1200,7 @@
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="37" t="str">
-        <x:v>2. Fix the advertising decision loop: $50.6K of SKU-less ad cost consumes 98.7% of CM1; ingest campaign/SKU ad detail before scaling spend.</x:v>
+        <x:v>2. Fix the advertising decision loop: $50.6K of SKU-less ad cost consumes 98.7% of contribution margin; ingest campaign/SKU ad detail before scaling spend.</x:v>
       </x:c>
       <x:c r="B18" s="37"/>
       <x:c r="C18" s="37"/>
@@ -1220,7 +1220,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="74" t="str">
-        <x:v>Decision caveat: two SKUs (2.3% of gross sales) use brand-median cost. CM1 is decision-useful, but those costs should be replaced before final accounting. Platform overhead remains below CM1 because the supplied file lacks causal SKU keys.</x:v>
+        <x:v>Decision caveat: two SKUs (2.3% of gross sales) use brand-median cost. Their costs should be replaced before final accounting. Platform costs are shown after contribution margin because the supplied file lacks reliable SKU keys.</x:v>
       </x:c>
       <x:c r="B21" s="75"/>
       <x:c r="C21" s="75"/>
@@ -1262,7 +1262,7 @@
     <x:mergeCell ref="A21:F23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16d54cc3950744e8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb689ee4e27c44c94"/>
 </x:worksheet>
 </file>
 
@@ -1342,7 +1342,7 @@
         <x:v>Contribution Margin</x:v>
       </x:c>
       <x:c r="J4" s="14" t="str">
-        <x:v>CM %</x:v>
+        <x:v>Margin %</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1515,7 +1515,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68842b23e5fa4fc0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c28a3ec8b90479e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1576,7 +1576,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>CM1 = net sales after promotions - referral fees - FBA fees - landed COGS</x:v>
+        <x:v>Contribution margin = net sales after promotions - referral fees - FBA fees - landed COGS</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
@@ -1620,7 +1620,7 @@
         <x:v>Contribution Margin</x:v>
       </x:c>
       <x:c r="N4" s="14" t="str">
-        <x:v>CM %</x:v>
+        <x:v>Margin %</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -2796,7 +2796,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6ad61b3be8c4ceb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra25a5de25c7346e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4168,7 +4168,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R625ea1bc57d947e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd681b122bf85405c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4301,7 +4301,7 @@
         <x:v>9 settlement rows lack SKU, including advertising, storage, and subscription fees.</x:v>
       </x:c>
       <x:c r="D9" s="32" t="str">
-        <x:v>Kept these amounts below SKU-attributable CM1; did not force an allocation.</x:v>
+        <x:v>Kept these amounts below SKU-attributable contribution margin; did not force an allocation.</x:v>
       </x:c>
       <x:c r="E9" s="32" t="str">
         <x:v>Ingest advertising campaign/product reports and storage SKU detail before allocation.</x:v>
@@ -4378,7 +4378,7 @@
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
       <x:c r="A17" s="37" t="str">
-        <x:v>• Advertising, storage, subscription, and adjustments stay below CM1 because they lack a defensible SKU allocation key.</x:v>
+        <x:v>• Advertising, storage, subscription, and adjustments are shown separately because they lack a reliable SKU allocation key.</x:v>
       </x:c>
       <x:c r="B17" s="37"/>
       <x:c r="C17" s="37"/>
@@ -4428,7 +4428,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b9307973a3349f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0de56707a24c4f9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5366,7 +5366,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00fb9fa0816a4d1b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R128e773e22e04e7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5434,7 +5434,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Brand CM ties to SKU CM</x:v>
+        <x:v>Brand contribution margin ties to SKU detail</x:v>
       </x:c>
       <x:c r="B5" s="38" t="n">
         <x:f>SUM('Brand Profitability'!I5:I7)</x:f>

</xml_diff>

<commit_message>
Organize source files and finalize audit fixes
</commit_message>
<xml_diff>
--- a/deliverables/Amazon_Q2_2026_Profitability_Analysis.xlsx
+++ b/deliverables/Amazon_Q2_2026_Profitability_Analysis.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R43576ba2c2d2418e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Profitability" sheetId="2" r:id="R2079f288094f490b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKU Profitability" sheetId="3" r:id="R82114d1812d5459a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory Health" sheetId="4" r:id="Rccedbad2bf044ab2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQ &amp; Assumptions" sheetId="5" r:id="R296876f5914a4c97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PO Unit Costs" sheetId="6" r:id="R4a422f2adc6f4bea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="7" r:id="Rb9cdfe3e79be41ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R917d685a60f3409a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Profitability" sheetId="2" r:id="Rb491356bc0214534"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKU Profitability" sheetId="3" r:id="R5a51d7b0149a40f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory Health" sheetId="4" r:id="R89b90e820d12473a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQ &amp; Assumptions" sheetId="5" r:id="R658fac9e70714d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PO Unit Costs" sheetId="6" r:id="Rcaa47b26e7c74b3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="7" r:id="Rd739bee0cfea48ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -402,7 +402,7 @@
         <x:color rgb="FF9A6700"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -413,7 +413,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -424,7 +424,7 @@
         <x:color rgb="FF9A6700"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -435,7 +435,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -446,7 +446,7 @@
         <x:color rgb="FF9A6700"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -457,7 +457,7 @@
         <x:color rgb="FF0B7A53"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD1FAE5"/>
         </x:patternFill>
       </x:fill>
@@ -468,7 +468,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -618,7 +618,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0798236d84c44e60"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R00d9861a06f8496e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1200,7 +1200,7 @@
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="37" t="str">
-        <x:v>2. Fix the advertising decision loop: $50.6K of SKU-less ad cost consumes 98.7% of contribution margin; ingest campaign/SKU ad detail before scaling spend.</x:v>
+        <x:v>2. Set a provisional $38.4K quarterly ad guardrail for a 5% post-platform margin; reallocate using campaign/ASIN contribution data.</x:v>
       </x:c>
       <x:c r="B18" s="37"/>
       <x:c r="C18" s="37"/>
@@ -1262,7 +1262,7 @@
     <x:mergeCell ref="A21:F23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb689ee4e27c44c94"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ee71356a44d40c6"/>
 </x:worksheet>
 </file>
 
@@ -1515,7 +1515,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c28a3ec8b90479e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb29f2c2f40274b0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2796,7 +2796,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra25a5de25c7346e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ab8a46f98e445a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4168,7 +4168,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd681b122bf85405c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f7d94683ca84429"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4295,13 +4295,13 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="B9" s="32" t="str">
-        <x:v>Platform fees and adjustments have no usable SKU allocation key</x:v>
+        <x:v>Shared platform costs lack SKU keys; adjustments lack accounting detail</x:v>
       </x:c>
       <x:c r="C9" s="32" t="str">
-        <x:v>9 settlement rows lack SKU, including advertising, storage, and subscription fees.</x:v>
+        <x:v>9 advertising/storage/subscription rows lack SKU; 2 adjustment rows have SKU but no reason or accounting treatment.</x:v>
       </x:c>
       <x:c r="D9" s="32" t="str">
-        <x:v>Kept these amounts below SKU-attributable contribution margin; did not force an allocation.</x:v>
+        <x:v>Kept both below SKU contribution margin; allocated only shared platform costs in the threshold check.</x:v>
       </x:c>
       <x:c r="E9" s="32" t="str">
         <x:v>Ingest advertising campaign/product reports and storage SKU detail before allocation.</x:v>
@@ -4315,10 +4315,10 @@
         <x:v>PO data has no receipt/status lifecycle</x:v>
       </x:c>
       <x:c r="C10" s="32" t="str">
-        <x:v>PO date and inbound snapshot cannot prove whether a PO is open, shipped, received, or canceled.</x:v>
+        <x:v>PO date does not prove receipt/status; one post-quarter line (PO-2026-0183) was excluded.</x:v>
       </x:c>
       <x:c r="D10" s="32" t="str">
-        <x:v>Used PO lines only for weighted landed unit cost; did not label PO quantities as inbound.</x:v>
+        <x:v>Used available PO lines dated through June 30 for weighted cost; did not label PO quantities as inbound.</x:v>
       </x:c>
       <x:c r="E10" s="32" t="str">
         <x:v>Add PO header/status, expected ship/arrival, receipt, and Amazon shipment IDs.</x:v>
@@ -4378,7 +4378,7 @@
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
       <x:c r="A17" s="37" t="str">
-        <x:v>• Advertising, storage, subscription, and adjustments are shown separately because they lack a reliable SKU allocation key.</x:v>
+        <x:v>• Shared platform costs lack SKU keys; adjustments remain separate because their accounting purpose is unknown.</x:v>
       </x:c>
       <x:c r="B17" s="37"/>
       <x:c r="C17" s="37"/>
@@ -4428,7 +4428,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0de56707a24c4f9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a0ed5b5962c4094"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4483,7 +4483,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Weighted average landed cost; PH-DENTAL-30CT converted from cases at 12 units per case</x:v>
+        <x:v>Weighted average landed cost from available PO records dated through 2026-06-30; PH-DENTAL-30CT converted at 12 units per case</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
@@ -5181,31 +5181,31 @@
         <x:v>PawHaus Double-Sided Grooming Brush</x:v>
       </x:c>
       <x:c r="D22" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E22" s="31" t="n">
         <x:v>46092</x:v>
       </x:c>
       <x:c r="F22" s="31" t="n">
-        <x:v>46205</x:v>
+        <x:v>46092</x:v>
       </x:c>
       <x:c r="G22" s="17" t="n">
-        <x:v>600</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="H22" s="15" t="n">
-        <x:v>1434</x:v>
+        <x:v>956</x:v>
       </x:c>
       <x:c r="I22" s="15" t="n">
-        <x:v>124.80000000000001</x:v>
+        <x:v>83.2</x:v>
       </x:c>
       <x:c r="J22" s="15" t="n">
-        <x:v>1558.8000000000002</x:v>
+        <x:v>1039.2</x:v>
       </x:c>
       <x:c r="K22" s="17" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L22" s="16" t="n">
-        <x:v>2.5980000000000003</x:v>
+        <x:v>2.598</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -5366,7 +5366,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R128e773e22e04e7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb26476457e10464a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5591,7 +5591,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>Source arithmetic reconciles within floating-point tolerance</x:v>
+        <x:v>Source arithmetic reconciles; the July 2 PO is excluded from Q2 costing</x:v>
       </x:c>
     </x:row>
     <x:row r="12">

</xml_diff>

<commit_message>
Make profitability findings decision-ready
</commit_message>
<xml_diff>
--- a/deliverables/Amazon_Q2_2026_Profitability_Analysis.xlsx
+++ b/deliverables/Amazon_Q2_2026_Profitability_Analysis.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R917d685a60f3409a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Profitability" sheetId="2" r:id="Rb491356bc0214534"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKU Profitability" sheetId="3" r:id="R5a51d7b0149a40f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory Health" sheetId="4" r:id="R89b90e820d12473a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQ &amp; Assumptions" sheetId="5" r:id="R658fac9e70714d5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PO Unit Costs" sheetId="6" r:id="Rcaa47b26e7c74b3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="7" r:id="Rd739bee0cfea48ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Raa1f8f02eaea40ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Profitability" sheetId="2" r:id="R99d75d9a97c7430c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKU Profitability" sheetId="3" r:id="Rb7dec95c51084ecf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory Health" sheetId="4" r:id="Rec6f9446ad2845e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQ &amp; Assumptions" sheetId="5" r:id="R1d82543656ca433e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PO Unit Costs" sheetId="6" r:id="R08ddf4d4bc7f4883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="7" r:id="Rcccba539c6294368"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -618,7 +618,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R00d9861a06f8496e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re9e004e6248c431e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1190,7 +1190,7 @@
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="37" t="str">
-        <x:v>1. Protect profitable demand: Peak Fuel and GlowTheory generate 83% of contribution margin; GT-SERUM-VITC and PF-WHEY-CHOC are the largest SKU contributors.</x:v>
+        <x:v>1. Acquisition economics erase portfolio margin: 38.7% pre-ad CM falls to a $5.6K run-rate loss because advertising consumes 98.7% of CM. Use the $38.4K guardrail or deliver $12.2K more contribution.</x:v>
       </x:c>
       <x:c r="B17" s="37"/>
       <x:c r="C17" s="37"/>
@@ -1200,7 +1200,7 @@
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="37" t="str">
-        <x:v>2. Set a provisional $38.4K quarterly ad guardrail for a 5% post-platform margin; reallocate using campaign/ASIN contribution data.</x:v>
+        <x:v>2. PawHaus needs an economic decision: 25.6% reported CM and (17.3%) under the directional threshold; reprice, reduce dimensional weight, test FBM, or exit products below the margin floor.</x:v>
       </x:c>
       <x:c r="B18" s="37"/>
       <x:c r="C18" s="37"/>
@@ -1210,7 +1210,7 @@
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="37" t="str">
-        <x:v>3. Rebalance inventory: PF-WHEY-CHOC and GT-SERUM-VITC have &lt;60 days of fulfillable cover, while 13 SKUs exceed one year of cover at Q2 demand.</x:v>
+        <x:v>3. Advertising attribution determines what to cut: ingest campaign and advertised-ASIN spend to identify whether losses are broad or concentrated; manage contribution after ads, not ROAS alone.</x:v>
       </x:c>
       <x:c r="B19" s="37"/>
       <x:c r="C19" s="37"/>
@@ -1220,7 +1220,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="74" t="str">
-        <x:v>Decision caveat: two SKUs (2.3% of gross sales) use brand-median cost. Their costs should be replaced before final accounting. Platform costs are shown after contribution margin because the supplied file lacks reliable SKU keys.</x:v>
+        <x:v>Validation next steps: replace two imputed costs; add receipt-layer costing and inventory movements; match returns to cohorts and disposition. Platform costs remain below SKU CM until product keys are available.</x:v>
       </x:c>
       <x:c r="B21" s="75"/>
       <x:c r="C21" s="75"/>
@@ -1262,7 +1262,7 @@
     <x:mergeCell ref="A21:F23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ee71356a44d40c6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3348b4f88a141f9"/>
 </x:worksheet>
 </file>
 
@@ -1515,7 +1515,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb29f2c2f40274b0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88b932c365dc4bb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2796,7 +2796,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ab8a46f98e445a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32d3081b7f034786"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4168,7 +4168,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f7d94683ca84429"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75b72f6c0a744b98"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4428,7 +4428,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a0ed5b5962c4094"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73439a9a2b524811"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5366,7 +5366,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb26476457e10464a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re05e1f4f23da4995"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>